<commit_message>
Leave status blank on spare schedule rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wt153oLhZWmCLgFgr6RgtT
</commit_message>
<xml_diff>
--- a/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
+++ b/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="322">
   <si>
     <r>
       <rPr>
@@ -5003,7 +5003,7 @@
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="2" t="str">
         <f aca="false">"未記入："&amp;COUNTIF(配信スケジュール!$P$3:$P$59,"未記入")&amp;" 通"</f>
-        <v>未記入：57 通</v>
+        <v>未記入：47 通</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6916,9 +6916,7 @@
       <c r="M50" s="17"/>
       <c r="N50" s="17"/>
       <c r="O50" s="17"/>
-      <c r="P50" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P50" s="18"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="13" t="n">
@@ -6941,9 +6939,7 @@
       <c r="M51" s="17"/>
       <c r="N51" s="17"/>
       <c r="O51" s="17"/>
-      <c r="P51" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P51" s="18"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="n">
@@ -6966,9 +6962,7 @@
       <c r="M52" s="17"/>
       <c r="N52" s="17"/>
       <c r="O52" s="17"/>
-      <c r="P52" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P52" s="18"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="13" t="n">
@@ -6991,9 +6985,7 @@
       <c r="M53" s="17"/>
       <c r="N53" s="17"/>
       <c r="O53" s="17"/>
-      <c r="P53" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P53" s="18"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="13" t="n">
@@ -7016,9 +7008,7 @@
       <c r="M54" s="17"/>
       <c r="N54" s="17"/>
       <c r="O54" s="17"/>
-      <c r="P54" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P54" s="18"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="13" t="n">
@@ -7041,9 +7031,7 @@
       <c r="M55" s="17"/>
       <c r="N55" s="17"/>
       <c r="O55" s="17"/>
-      <c r="P55" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P55" s="18"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="13" t="n">
@@ -7066,9 +7054,7 @@
       <c r="M56" s="17"/>
       <c r="N56" s="17"/>
       <c r="O56" s="17"/>
-      <c r="P56" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P56" s="18"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="13" t="n">
@@ -7091,9 +7077,7 @@
       <c r="M57" s="17"/>
       <c r="N57" s="17"/>
       <c r="O57" s="17"/>
-      <c r="P57" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P57" s="18"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="n">
@@ -7116,9 +7100,7 @@
       <c r="M58" s="17"/>
       <c r="N58" s="17"/>
       <c r="O58" s="17"/>
-      <c r="P58" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P58" s="18"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="13" t="n">
@@ -7141,9 +7123,7 @@
       <c r="M59" s="17"/>
       <c r="N59" s="17"/>
       <c r="O59" s="17"/>
-      <c r="P59" s="18" t="s">
-        <v>44</v>
-      </c>
+      <c r="P59" s="18"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P59"/>

</xml_diff>

<commit_message>
Fill participant bonus list (30 items) in LINE input sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wt153oLhZWmCLgFgr6RgtT
</commit_message>
<xml_diff>
--- a/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
+++ b/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
@@ -88,7 +88,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="D30" authorId="0">
+    <comment ref="D40" authorId="0">
       <text>
         <r>
           <rPr>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="360">
   <si>
     <r>
       <rPr>
@@ -3810,7 +3810,412 @@
     <t xml:space="preserve">参加特典</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IELTS 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">技能 現在地診断シート</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">【診断・分析】</t>
+  </si>
+  <si>
+    <t xml:space="preserve">シート</t>
+  </si>
+  <si>
     <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">スコアレポート分析シート</t>
+  </si>
+  <si>
+    <t xml:space="preserve">今の勉強法チェックリスト</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">停滞する人のパターン</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">時間の棚卸しシート</t>
+  </si>
+  <si>
+    <t xml:space="preserve">目標の言語化シート</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">半年で</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+1.0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">逆算ロードマップ</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">【計画・記録】</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">週間計画</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">振り返りシート</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">学習ログシート</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">模試計画</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">スコア推移シート</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">試験日逆算カレンダー</t>
+  </si>
+  <si>
+    <t xml:space="preserve">次アクションシート</t>
+  </si>
+  <si>
+    <t xml:space="preserve">採点基準の読み方ガイド</t>
+  </si>
+  <si>
+    <t xml:space="preserve">【ライティング】</t>
+  </si>
+  <si>
+    <t xml:space="preserve">自己添削チェックリスト</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">添削ログ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">間違いノート</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">シート</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">と</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の答案比較解剖資料</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">アイデア発想法ガイド</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ライティング練習の組み方ガイド</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">T/F/NG </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">判定フローチャート</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">【リーディング・リスニング】</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">解く順</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">時間配分ガイド</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">間違い原因分類シート</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ディクテーション</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日間メニュー</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">シャドーイング段階別ガイド</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ひとりスピーキング練習メニュー</t>
+  </si>
+  <si>
+    <t xml:space="preserve">【スピーキング】</t>
+  </si>
+  <si>
+    <t xml:space="preserve">スピーキング失点セルフ分析シート</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Part 2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">準備</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分の考え方ガイド</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">習慣設計ガイド</t>
+  </si>
+  <si>
+    <t xml:space="preserve">【継続・導線】</t>
+  </si>
+  <si>
+    <t xml:space="preserve">挫折分岐シート</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">週間お試しコーチング体験券</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">招待・体験</t>
+  </si>
+  <si>
+    <t xml:space="preserve">コミュニティ招待券</t>
   </si>
   <si>
     <t xml:space="preserve">参加特典の数（自動）</t>
@@ -7831,7 +8236,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -8006,11 +8411,17 @@
       <c r="B9" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
+      <c r="C9" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F9" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G9" s="17"/>
     </row>
@@ -8021,11 +8432,17 @@
       <c r="B10" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
+      <c r="C10" s="18" t="s">
+        <v>265</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F10" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G10" s="17"/>
     </row>
@@ -8036,11 +8453,17 @@
       <c r="B11" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
+      <c r="C11" s="18" t="s">
+        <v>266</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F11" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G11" s="17"/>
     </row>
@@ -8051,11 +8474,17 @@
       <c r="B12" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
+      <c r="C12" s="18" t="s">
+        <v>267</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F12" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G12" s="17"/>
     </row>
@@ -8066,11 +8495,17 @@
       <c r="B13" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
+      <c r="C13" s="18" t="s">
+        <v>268</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F13" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G13" s="17"/>
     </row>
@@ -8081,11 +8516,17 @@
       <c r="B14" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
+      <c r="C14" s="18" t="s">
+        <v>269</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>262</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F14" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G14" s="17"/>
     </row>
@@ -8096,11 +8537,17 @@
       <c r="B15" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
+      <c r="C15" s="18" t="s">
+        <v>270</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F15" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G15" s="17"/>
     </row>
@@ -8111,11 +8558,17 @@
       <c r="B16" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
+      <c r="C16" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F16" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G16" s="17"/>
     </row>
@@ -8126,11 +8579,17 @@
       <c r="B17" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
+      <c r="C17" s="18" t="s">
+        <v>273</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F17" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G17" s="17"/>
     </row>
@@ -8141,11 +8600,17 @@
       <c r="B18" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
+      <c r="C18" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F18" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G18" s="17"/>
     </row>
@@ -8156,11 +8621,17 @@
       <c r="B19" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
+      <c r="C19" s="18" t="s">
+        <v>275</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F19" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G19" s="17"/>
     </row>
@@ -8171,11 +8642,17 @@
       <c r="B20" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
+      <c r="C20" s="18" t="s">
+        <v>276</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>271</v>
+      </c>
+      <c r="E20" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F20" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G20" s="17"/>
     </row>
@@ -8186,11 +8663,17 @@
       <c r="B21" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
+      <c r="C21" s="18" t="s">
+        <v>277</v>
+      </c>
+      <c r="D21" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F21" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G21" s="17"/>
     </row>
@@ -8201,11 +8684,17 @@
       <c r="B22" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
+      <c r="C22" s="18" t="s">
+        <v>279</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F22" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G22" s="17"/>
     </row>
@@ -8216,11 +8705,17 @@
       <c r="B23" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
+      <c r="C23" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="F23" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G23" s="17"/>
     </row>
@@ -8231,11 +8726,17 @@
       <c r="B24" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
+      <c r="C24" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="D24" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F24" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G24" s="17"/>
     </row>
@@ -8246,11 +8747,17 @@
       <c r="B25" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
+      <c r="C25" s="18" t="s">
+        <v>282</v>
+      </c>
+      <c r="D25" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F25" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G25" s="17"/>
     </row>
@@ -8261,11 +8768,17 @@
       <c r="B26" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="C26" s="17"/>
-      <c r="D26" s="17"/>
-      <c r="E26" s="17"/>
+      <c r="C26" s="18" t="s">
+        <v>283</v>
+      </c>
+      <c r="D26" s="18" t="s">
+        <v>278</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F26" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G26" s="17"/>
     </row>
@@ -8276,11 +8789,17 @@
       <c r="B27" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="C27" s="17"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
+      <c r="C27" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="D27" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F27" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G27" s="17"/>
     </row>
@@ -8291,21 +8810,237 @@
       <c r="B28" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
+      <c r="C28" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="D28" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>247</v>
+      </c>
       <c r="F28" s="13" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G28" s="17"/>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B29" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="C29" s="18" t="s">
+        <v>287</v>
+      </c>
+      <c r="D29" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G29" s="17"/>
+    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C30" s="20" t="s">
-        <v>262</v>
-      </c>
-      <c r="D30" s="13" t="n">
-        <f aca="false">COUNTIFS(A3:A28,"参加特典",C3:C28,"&lt;&gt;")</f>
-        <v>0</v>
+      <c r="A30" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G30" s="17"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B31" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>289</v>
+      </c>
+      <c r="D31" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G31" s="17"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B32" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D32" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G32" s="17"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B33" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C33" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="D33" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E33" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G33" s="17"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B34" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>293</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>291</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G34" s="17"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B35" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="D35" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G35" s="17"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B36" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="C36" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="D36" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>263</v>
+      </c>
+      <c r="F36" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G36" s="17"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B37" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>297</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="E37" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="F37" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G37" s="17"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B38" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>264</v>
+      </c>
+      <c r="G38" s="17"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C40" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="D40" s="13" t="n">
+        <f aca="false">COUNTIFS(A3:A38,"参加特典",C3:C38,"&lt;&gt;")</f>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -8341,34 +9076,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>263</v>
+        <v>301</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>264</v>
+        <v>302</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>265</v>
+        <v>303</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>266</v>
+        <v>304</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>267</v>
+        <v>305</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>268</v>
+        <v>306</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>269</v>
+        <v>307</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>270</v>
+        <v>308</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>271</v>
+        <v>309</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>272</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8376,36 +9111,36 @@
         <v>32</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>273</v>
+        <v>311</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>274</v>
+        <v>312</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>275</v>
+        <v>313</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>276</v>
+        <v>314</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>277</v>
+        <v>315</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>278</v>
+        <v>316</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>279</v>
+        <v>317</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>280</v>
+        <v>318</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>281</v>
+        <v>319</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>282</v>
+        <v>320</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -8419,7 +9154,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>283</v>
+        <v>321</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -8433,7 +9168,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>284</v>
+        <v>322</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -8447,7 +9182,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>285</v>
+        <v>323</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -8461,7 +9196,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>286</v>
+        <v>324</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -8475,7 +9210,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>287</v>
+        <v>325</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -8489,7 +9224,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>288</v>
+        <v>326</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -8503,7 +9238,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>289</v>
+        <v>327</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -8551,25 +9286,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>290</v>
+        <v>328</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>291</v>
+        <v>329</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>292</v>
+        <v>330</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>293</v>
+        <v>331</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>294</v>
+        <v>332</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>295</v>
+        <v>333</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>296</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8577,27 +9312,27 @@
         <v>32</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>297</v>
+        <v>335</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>298</v>
+        <v>336</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>299</v>
+        <v>337</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>300</v>
+        <v>338</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>227</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>301</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>302</v>
+        <v>340</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -8608,7 +9343,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>303</v>
+        <v>341</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -8619,7 +9354,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>304</v>
+        <v>342</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -8630,7 +9365,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>305</v>
+        <v>343</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -8641,7 +9376,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>306</v>
+        <v>344</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -8652,7 +9387,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>307</v>
+        <v>345</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -8663,7 +9398,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>308</v>
+        <v>346</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -8674,7 +9409,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>309</v>
+        <v>347</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -8685,7 +9420,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>310</v>
+        <v>348</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -8696,7 +9431,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>311</v>
+        <v>349</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -8707,7 +9442,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>312</v>
+        <v>350</v>
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -8718,7 +9453,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>313</v>
+        <v>351</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -8729,7 +9464,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>314</v>
+        <v>352</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -8740,7 +9475,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>315</v>
+        <v>353</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -8751,7 +9486,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>316</v>
+        <v>354</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -8762,7 +9497,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>317</v>
+        <v>355</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -8773,7 +9508,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>318</v>
+        <v>356</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -8784,7 +9519,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>319</v>
+        <v>357</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -8795,7 +9530,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>320</v>
+        <v>358</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -8806,7 +9541,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>321</v>
+        <v>359</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>

</xml_diff>

<commit_message>
Update bonus list: merge overlaps, sharpen titles, add AI prompt bonuses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wt153oLhZWmCLgFgr6RgtT
</commit_message>
<xml_diff>
--- a/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
+++ b/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="361">
   <si>
     <r>
       <rPr>
@@ -3863,7 +3863,48 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">時間の棚卸しシート</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">社会人が</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">時間をつくる 時間の棚卸しシート</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">目標の言語化シート</t>
@@ -3892,7 +3933,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">逆算ロードマップ</t>
+      <t xml:space="preserve">逆算ロードマップ（試験日逆算カレンダー付き）</t>
     </r>
   </si>
   <si>
@@ -3922,11 +3963,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">振り返りシート</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">学習ログシート</t>
+      <t xml:space="preserve">学習ログシート</t>
+    </r>
   </si>
   <si>
     <r>
@@ -3956,13 +3994,10 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">試験日逆算カレンダー</t>
-  </si>
-  <si>
     <t xml:space="preserve">次アクションシート</t>
   </si>
   <si>
-    <t xml:space="preserve">採点基準の読み方ガイド</t>
+    <t xml:space="preserve">試験官はここを見ている 採点基準の読み方ガイド</t>
   </si>
   <si>
     <t xml:space="preserve">【ライティング】</t>
@@ -4051,7 +4086,40 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">アイデア発想法ガイド</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Task 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で手が止まらない アイデア発想法</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">パターン</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">ライティング練習の組み方ガイド</t>
@@ -4106,7 +4174,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">間違い原因分類シート</t>
+    <t xml:space="preserve">「なんとなく間違えた」をなくす 間違い原因分類シート</t>
   </si>
   <si>
     <r>
@@ -4139,7 +4207,57 @@
     <t xml:space="preserve">シャドーイング段階別ガイド</t>
   </si>
   <si>
-    <t xml:space="preserve">ひとりスピーキング練習メニュー</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分 ひとりスピーキング練習メニュー</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日分</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">【スピーキング】</t>
@@ -4184,15 +4302,164 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">習慣設計ガイド</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を試験官にする </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Speaking</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">模擬試験プロンプト集</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">【</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">活用】</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Writing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">自己添削 プロンプト集（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Task 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で自分専用の単語帳をつくる プロンプト集</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">習慣設計＆挫折分岐ガイド</t>
   </si>
   <si>
     <t xml:space="preserve">【継続・導線】</t>
   </si>
   <si>
-    <t xml:space="preserve">挫折分岐シート</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -4208,7 +4475,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">週間お試しコーチング体験券</t>
+      <t xml:space="preserve">週間お試しコーチング体験券（先着○名）</t>
     </r>
   </si>
   <si>
@@ -8530,7 +8797,7 @@
       </c>
       <c r="G14" s="17"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
         <v>260</v>
       </c>
@@ -8614,7 +8881,7 @@
       </c>
       <c r="G18" s="17"/>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
         <v>260</v>
       </c>
@@ -8625,10 +8892,10 @@
         <v>275</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>271</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>263</v>
+        <v>276</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>247</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>264</v>
@@ -8643,13 +8910,13 @@
         <v>12</v>
       </c>
       <c r="C20" s="18" t="s">
+        <v>277</v>
+      </c>
+      <c r="D20" s="18" t="s">
         <v>276</v>
       </c>
-      <c r="D20" s="18" t="s">
-        <v>271</v>
-      </c>
-      <c r="E20" s="18" t="s">
-        <v>263</v>
+      <c r="E20" s="17" t="s">
+        <v>247</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>264</v>
@@ -8664,13 +8931,13 @@
         <v>13</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>278</v>
-      </c>
-      <c r="E21" s="17" t="s">
-        <v>247</v>
+        <v>276</v>
+      </c>
+      <c r="E21" s="18" t="s">
+        <v>263</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>264</v>
@@ -8684,11 +8951,11 @@
       <c r="B22" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="17" t="s">
         <v>279</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>247</v>
@@ -8698,21 +8965,21 @@
       </c>
       <c r="G22" s="17"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
         <v>260</v>
       </c>
       <c r="B23" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="17" t="s">
         <v>280</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>278</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>263</v>
+        <v>276</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>247</v>
       </c>
       <c r="F23" s="13" t="s">
         <v>264</v>
@@ -8726,11 +8993,11 @@
       <c r="B24" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="18" t="s">
         <v>281</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>247</v>
@@ -8747,11 +9014,11 @@
       <c r="B25" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="17" t="s">
         <v>282</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="E25" s="17" t="s">
         <v>247</v>
@@ -8769,10 +9036,10 @@
         <v>18</v>
       </c>
       <c r="C26" s="18" t="s">
+        <v>284</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>283</v>
-      </c>
-      <c r="D26" s="18" t="s">
-        <v>278</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>247</v>
@@ -8782,21 +9049,21 @@
       </c>
       <c r="G26" s="17"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
         <v>260</v>
       </c>
       <c r="B27" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="C27" s="17" t="s">
-        <v>284</v>
+      <c r="C27" s="18" t="s">
+        <v>285</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="E27" s="17" t="s">
-        <v>247</v>
+        <v>283</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>263</v>
       </c>
       <c r="F27" s="13" t="s">
         <v>264</v>
@@ -8814,7 +9081,7 @@
         <v>286</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E28" s="17" t="s">
         <v>247</v>
@@ -8835,28 +9102,28 @@
         <v>287</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="E29" s="18" t="s">
-        <v>263</v>
+        <v>283</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>247</v>
       </c>
       <c r="F29" s="13" t="s">
         <v>264</v>
       </c>
       <c r="G29" s="17"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
         <v>260</v>
       </c>
       <c r="B30" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C30" s="17" t="s">
         <v>288</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>247</v>
@@ -8874,13 +9141,13 @@
         <v>23</v>
       </c>
       <c r="C31" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D31" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="D31" s="18" t="s">
-        <v>285</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>247</v>
+      <c r="E31" s="18" t="s">
+        <v>263</v>
       </c>
       <c r="F31" s="13" t="s">
         <v>264</v>
@@ -8894,11 +9161,11 @@
       <c r="B32" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="C32" s="18" t="s">
-        <v>290</v>
+      <c r="C32" s="17" t="s">
+        <v>291</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="E32" s="17" t="s">
         <v>247</v>
@@ -8908,28 +9175,28 @@
       </c>
       <c r="G32" s="17"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
         <v>260</v>
       </c>
       <c r="B33" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="C33" s="18" t="s">
+      <c r="C33" s="17" t="s">
         <v>292</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="E33" s="18" t="s">
-        <v>263</v>
+        <v>293</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>247</v>
       </c>
       <c r="F33" s="13" t="s">
         <v>264</v>
       </c>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
         <v>260</v>
       </c>
@@ -8937,10 +9204,10 @@
         <v>26</v>
       </c>
       <c r="C34" s="17" t="s">
+        <v>294</v>
+      </c>
+      <c r="D34" s="18" t="s">
         <v>293</v>
-      </c>
-      <c r="D34" s="18" t="s">
-        <v>291</v>
       </c>
       <c r="E34" s="17" t="s">
         <v>247</v>
@@ -8957,11 +9224,11 @@
       <c r="B35" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="C35" s="18" t="s">
-        <v>294</v>
+      <c r="C35" s="17" t="s">
+        <v>295</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="E35" s="17" t="s">
         <v>247</v>
@@ -8982,10 +9249,10 @@
         <v>296</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="E36" s="18" t="s">
-        <v>263</v>
+        <v>297</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>247</v>
       </c>
       <c r="F36" s="13" t="s">
         <v>264</v>
@@ -9000,13 +9267,13 @@
         <v>29</v>
       </c>
       <c r="C37" s="17" t="s">
+        <v>298</v>
+      </c>
+      <c r="D37" s="18" t="s">
         <v>297</v>
       </c>
-      <c r="D37" s="18" t="s">
-        <v>295</v>
-      </c>
       <c r="E37" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F37" s="13" t="s">
         <v>264</v>
@@ -9021,13 +9288,13 @@
         <v>30</v>
       </c>
       <c r="C38" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="E38" s="18" t="s">
         <v>299</v>
-      </c>
-      <c r="D38" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="E38" s="18" t="s">
-        <v>298</v>
       </c>
       <c r="F38" s="13" t="s">
         <v>264</v>
@@ -9036,7 +9303,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C40" s="20" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D40" s="13" t="n">
         <f aca="false">COUNTIFS(A3:A38,"参加特典",C3:C38,"&lt;&gt;")</f>
@@ -9076,34 +9343,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9111,36 +9378,36 @@
         <v>32</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -9154,7 +9421,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -9168,7 +9435,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -9182,7 +9449,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -9196,7 +9463,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -9210,7 +9477,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -9224,7 +9491,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -9238,7 +9505,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -9286,25 +9553,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9312,27 +9579,27 @@
         <v>32</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>227</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -9343,7 +9610,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -9354,7 +9621,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -9365,7 +9632,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -9376,7 +9643,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -9387,7 +9654,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -9398,7 +9665,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -9409,7 +9676,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -9420,7 +9687,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -9431,7 +9698,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -9442,7 +9709,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -9453,7 +9720,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -9464,7 +9731,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -9475,7 +9742,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -9486,7 +9753,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -9497,7 +9764,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -9508,7 +9775,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -9519,7 +9786,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -9530,7 +9797,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -9541,7 +9808,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>

</xml_diff>

<commit_message>
Add tentative contents for all bonuses in LINE input sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wt153oLhZWmCLgFgr6RgtT
</commit_message>
<xml_diff>
--- a/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
+++ b/line_campaign/12月勉強会_LINE配信_入力シート.xlsx
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="390">
   <si>
     <r>
       <rPr>
@@ -3671,6 +3671,33 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）社会人から</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IELTS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">に挑戦し、人生が変わった自分のストーリー</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">音声</t>
   </si>
   <si>
@@ -3721,6 +3748,50 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年にスコアを取り切るために、まず決めるべき</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">つのこと</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">12/11</t>
   </si>
   <si>
@@ -3751,12 +3822,42 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）多くの人が気づかずにハマる</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">つの落とし穴と抜け出し方</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">12/12</t>
   </si>
   <si>
     <t xml:space="preserve">○名以上を指導して分かったスコアアップの本当のカギ</t>
   </si>
   <si>
+    <t xml:space="preserve">（仮）たくさんの受講生を見てきて分かった、伸びる人の共通点</t>
+  </si>
+  <si>
     <t xml:space="preserve">12/15</t>
   </si>
   <si>
@@ -3804,9 +3905,73 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">時代でも</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IELTS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・英語を学ぶ価値と、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">との付き合い方</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">いちばん伝えたいメッセージ</t>
   </si>
   <si>
+    <t xml:space="preserve">（仮）勉強会の前に、いちばん伝えたい想い</t>
+  </si>
+  <si>
     <t xml:space="preserve">参加特典</t>
   </si>
   <si>
@@ -3829,7 +3994,48 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">【診断・分析】</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【診断・分析】各技能の今のスコア・目標・得意</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">苦手を書き出し、どこから伸ばすかを</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">枚で見える化。勉強会当日のワークでも使用</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">シート</t>
@@ -3841,6 +4047,9 @@
     <t xml:space="preserve">スコアレポート分析シート</t>
   </si>
   <si>
+    <t xml:space="preserve">（仮）【診断・分析】公式スコアレポートの数字から、どの技能・どの採点項目が足を引っ張っているかを読み解く記入式シート</t>
+  </si>
+  <si>
     <t xml:space="preserve">今の勉強法チェックリスト</t>
   </si>
   <si>
@@ -3850,6 +4059,33 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">（仮）【診断・分析】今の勉強が「スコアにつながる勉強」になっているかを</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">項目でセルフチェック</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">停滞する人のパターン</t>
     </r>
     <r>
@@ -3869,6 +4105,67 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">（仮）【診断・分析】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で止まる人に共通する</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の勉強パターンと、それぞれの抜け出し方</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">社会人が</t>
     </r>
     <r>
@@ -3907,6 +4204,33 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【診断・分析】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">週間の時間の使い方を書き出し、勉強に回せるすき間時間を見つける</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">目標の言語化シート</t>
   </si>
   <si>
@@ -3916,6 +4240,33 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">（仮）【診断・分析】「なぜ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">IELTS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">か」「いつまでに何点か」「取れたら何をするか」を言葉にして、続ける理由をつくる</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">半年で</t>
     </r>
     <r>
@@ -3937,7 +4288,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">【計画・記録】</t>
+    <t xml:space="preserve">（仮）【計画・記録】試験日から逆算して、月ごと・週ごとにやることを決めるロードマップ。カレンダーに書き込んで使う</t>
   </si>
   <si>
     <r>
@@ -3973,6 +4324,50 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">（仮）【計画・記録】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">週間の計画と、毎日の学習記録・振り返りを</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">枚で管理</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">模試計画</t>
     </r>
     <r>
@@ -3994,13 +4389,84 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">（仮）【計画・記録】模試をいつ解くかの計画と、技能別スコアの推移をグラフで記録</t>
+  </si>
+  <si>
     <t xml:space="preserve">次アクションシート</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【計画・記録】勉強会で学んだことから、明日からの具体的な行動を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">つに絞って書き出す（勉強会の最後に使用）</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">試験官はここを見ている 採点基準の読み方ガイド</t>
   </si>
   <si>
-    <t xml:space="preserve">【ライティング】</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【ライティング】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Writing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">つの採点基準（課題達成・一貫性・語彙・文法）を、日本人向けにかみくだいて解説</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">自己添削チェックリスト</t>
@@ -4012,6 +4478,33 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">（仮）【ライティング】書き終わった答案を自分で見直すためのチェック項目。採点基準の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">項目ごとに整理</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">添削ログ</t>
     </r>
     <r>
@@ -4050,6 +4543,9 @@
     </r>
   </si>
   <si>
+    <t xml:space="preserve">（仮）【ライティング】添削で指摘されたミスを種類ごとに記録し、同じミスを繰り返さないための記録シート</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -4089,6 +4585,67 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【ライティング】同じ設問の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">答案と</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6.5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">答案を並べ、どこで点差がついたかを</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">文ずつ解説</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -4122,12 +4679,66 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【ライティング】設問を見て意見・理由・具体例を素早く出すための考え方</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">つ（答え・例文は載せない）</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">ライティング練習の組み方ガイド</t>
   </si>
   <si>
     <r>
       <rPr>
         <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【ライティング】時間を計って書く→見直す→書き直す、の練習サイクルと</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">週間の回し方</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -4144,7 +4755,31 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">【リーディング・リスニング】</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【リーディング・リスニング】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">True / False / Not Given </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">を迷わず判定するための手順をフローチャートで</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4174,9 +4809,56 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【リーディング・リスニング】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Reading</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Listening</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">で、どの順番で解き、どこに何分かけるかの考え方</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">「なんとなく間違えた」をなくす 間違い原因分類シート</t>
   </si>
   <si>
+    <t xml:space="preserve">（仮）【リーディング・リスニング】間違えた問題を「単語」「文構造」「設問の読み違い」など原因別に分類し、弱点を特定する</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -4204,9 +4886,107 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【リーディング・リスニング】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Listening</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">力を上げるディクテーションを、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日間のメニューに</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">シャドーイング段階別ガイド</t>
   </si>
   <si>
+    <t xml:space="preserve">（仮）【リーディング・リスニング】聞く→つぶやく→重ねる→シャドーイング、と段階を踏んで進めるやり方と素材の選び方</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="10"/>
@@ -4260,7 +5040,82 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">【スピーキング】</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【スピーキング】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">人でできるスピーキング練習を、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">×30</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日分のメニューに（お題のみ・回答例なし）</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">スピーキング失点セルフ分析シート</t>
@@ -4269,6 +5124,33 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【スピーキング】自分の回答を録音して聞き直し、採点基準の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">項目ごとに失点ポイントを書き出す</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -4305,6 +5187,33 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【スピーキング】トピックカードを見てから話し始めるまでの</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">分間で、何をメモし、どう組み立てるか</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -4344,7 +5253,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">【</t>
+      <t xml:space="preserve">（仮）【</t>
     </r>
     <r>
       <rPr>
@@ -4363,6 +5272,57 @@
       </rPr>
       <t xml:space="preserve">活用】</t>
     </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ChatGPT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">等に試験官役をさせ、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Part 1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の模擬面接とフィードバックを受けるためのプロンプト集</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4438,6 +5398,14 @@
     <r>
       <rPr>
         <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -4450,14 +5418,94 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">活用】自分の答案を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">に読ませ、採点基準の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">項目ごとに弱点を指摘してもらうプロンプト集（スコア判定ではなく弱点発見用）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">で自分専用の単語帳をつくる プロンプト集</t>
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AI</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">活用】自分の答案や間違えた問題から、覚えるべき語彙を抜き出して単語帳にするプロンプト集</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">習慣設計＆挫折分岐ガイド</t>
   </si>
   <si>
-    <t xml:space="preserve">【継続・導線】</t>
+    <t xml:space="preserve">（仮）【継続・導線】勉強を習慣にする仕組みと、「忙しい」「伸びない」など挫折しそうな時の立て直し方</t>
   </si>
   <si>
     <r>
@@ -4479,10 +5527,40 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（仮）【継続・導線】</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">週間、学習計画へのアドバイスと進捗チェックを体験できる券（先着○名・人数は要決定）</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">招待・体験</t>
   </si>
   <si>
     <t xml:space="preserve">コミュニティ招待券</t>
+  </si>
+  <si>
+    <t xml:space="preserve">（仮）【継続・導線】一緒に学ぶ仲間とつながれるコミュニティへの招待（無料／有料・内容は要決定）</t>
   </si>
   <si>
     <t xml:space="preserve">参加特典の数（自動）</t>
@@ -8557,7 +9635,7 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
         <v>248</v>
       </c>
@@ -8567,12 +9645,14 @@
       <c r="C3" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="D3" s="17"/>
+      <c r="D3" s="18" t="s">
+        <v>250</v>
+      </c>
       <c r="E3" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G3" s="17"/>
     </row>
@@ -8584,18 +9664,20 @@
         <v>2</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="D4" s="17"/>
+        <v>253</v>
+      </c>
+      <c r="D4" s="18" t="s">
+        <v>254</v>
+      </c>
       <c r="E4" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="G4" s="17"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
         <v>248</v>
       </c>
@@ -8603,14 +9685,16 @@
         <v>3</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="D5" s="17"/>
+        <v>256</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>257</v>
+      </c>
       <c r="E5" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G5" s="17"/>
     </row>
@@ -8622,14 +9706,16 @@
         <v>4</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="D6" s="17"/>
+        <v>259</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>260</v>
+      </c>
       <c r="E6" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G6" s="17"/>
     </row>
@@ -8641,14 +9727,16 @@
         <v>5</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>258</v>
-      </c>
-      <c r="D7" s="17"/>
+        <v>262</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>263</v>
+      </c>
       <c r="E7" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F7" s="16" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G7" s="17"/>
     </row>
@@ -8660,650 +9748,652 @@
         <v>6</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="D8" s="17"/>
+        <v>264</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>265</v>
+      </c>
       <c r="E8" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="G8" s="17"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G9" s="17"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B10" s="16" t="n">
         <v>2</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G10" s="17"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>3</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="E11" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G11" s="17"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>4</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>262</v>
+        <v>276</v>
       </c>
       <c r="E12" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G12" s="17"/>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>5</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>262</v>
+        <v>278</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G13" s="17"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>6</v>
       </c>
       <c r="C14" s="18" t="s">
+        <v>279</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="E14" s="18" t="s">
         <v>269</v>
       </c>
-      <c r="D14" s="18" t="s">
-        <v>262</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>263</v>
-      </c>
       <c r="F14" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G14" s="17"/>
     </row>
-    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B15" s="16" t="n">
         <v>7</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>270</v>
+        <v>281</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>271</v>
+        <v>282</v>
       </c>
       <c r="E15" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G15" s="17"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B16" s="16" t="n">
         <v>8</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>272</v>
+        <v>283</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>271</v>
+        <v>284</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G16" s="17"/>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B17" s="16" t="n">
         <v>9</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F17" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G17" s="17"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B18" s="16" t="n">
         <v>10</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>274</v>
+        <v>287</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>271</v>
+        <v>288</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B19" s="16" t="n">
         <v>11</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>275</v>
+        <v>289</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>276</v>
+        <v>290</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G19" s="17"/>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B20" s="16" t="n">
         <v>12</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>277</v>
+        <v>291</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>276</v>
+        <v>292</v>
       </c>
       <c r="E20" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G20" s="17"/>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B21" s="16" t="n">
         <v>13</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>278</v>
+        <v>293</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G21" s="17"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B22" s="16" t="n">
         <v>14</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>276</v>
+        <v>296</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B23" s="16" t="n">
         <v>15</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>280</v>
+        <v>297</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>276</v>
+        <v>298</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G23" s="17"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B24" s="16" t="n">
         <v>16</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>276</v>
+        <v>300</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G24" s="17"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B25" s="16" t="n">
         <v>17</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="E25" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G25" s="17"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B26" s="16" t="n">
         <v>18</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>283</v>
+        <v>304</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G26" s="17"/>
     </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B27" s="16" t="n">
         <v>19</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>285</v>
+        <v>305</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>283</v>
+        <v>306</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G27" s="17"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B28" s="16" t="n">
         <v>20</v>
       </c>
       <c r="C28" s="18" t="s">
-        <v>286</v>
+        <v>307</v>
       </c>
       <c r="D28" s="18" t="s">
-        <v>283</v>
+        <v>308</v>
       </c>
       <c r="E28" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G28" s="17"/>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B29" s="16" t="n">
         <v>21</v>
       </c>
       <c r="C29" s="18" t="s">
-        <v>287</v>
+        <v>309</v>
       </c>
       <c r="D29" s="18" t="s">
-        <v>283</v>
+        <v>310</v>
       </c>
       <c r="E29" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B30" s="16" t="n">
         <v>22</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>288</v>
+        <v>311</v>
       </c>
       <c r="D30" s="18" t="s">
-        <v>289</v>
+        <v>312</v>
       </c>
       <c r="E30" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G30" s="17"/>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B31" s="16" t="n">
         <v>23</v>
       </c>
       <c r="C31" s="18" t="s">
-        <v>290</v>
+        <v>313</v>
       </c>
       <c r="D31" s="18" t="s">
-        <v>289</v>
+        <v>314</v>
       </c>
       <c r="E31" s="18" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G31" s="17"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B32" s="16" t="n">
         <v>24</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>291</v>
+        <v>315</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>289</v>
+        <v>316</v>
       </c>
       <c r="E32" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G32" s="17"/>
     </row>
     <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B33" s="16" t="n">
         <v>25</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>292</v>
+        <v>317</v>
       </c>
       <c r="D33" s="18" t="s">
-        <v>293</v>
+        <v>318</v>
       </c>
       <c r="E33" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F33" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G33" s="17"/>
     </row>
-    <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B34" s="16" t="n">
         <v>26</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>294</v>
+        <v>319</v>
       </c>
       <c r="D34" s="18" t="s">
-        <v>293</v>
+        <v>320</v>
       </c>
       <c r="E34" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F34" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G34" s="17"/>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B35" s="16" t="n">
         <v>27</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>295</v>
+        <v>321</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>293</v>
+        <v>322</v>
       </c>
       <c r="E35" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F35" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G35" s="17"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B36" s="16" t="n">
         <v>28</v>
       </c>
       <c r="C36" s="18" t="s">
-        <v>296</v>
+        <v>323</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>297</v>
+        <v>324</v>
       </c>
       <c r="E36" s="17" t="s">
         <v>247</v>
       </c>
       <c r="F36" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G36" s="17"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B37" s="16" t="n">
         <v>29</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>298</v>
+        <v>325</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>297</v>
+        <v>326</v>
       </c>
       <c r="E37" s="18" t="s">
-        <v>299</v>
+        <v>327</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G37" s="17"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B38" s="16" t="n">
         <v>30</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>300</v>
+        <v>328</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>297</v>
+        <v>329</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>299</v>
+        <v>327</v>
       </c>
       <c r="F38" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="G38" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C40" s="20" t="s">
-        <v>301</v>
+        <v>330</v>
       </c>
       <c r="D40" s="13" t="n">
         <f aca="false">COUNTIFS(A3:A38,"参加特典",C3:C38,"&lt;&gt;")</f>
@@ -9343,34 +10433,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>302</v>
+        <v>331</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>303</v>
+        <v>332</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>304</v>
+        <v>333</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>305</v>
+        <v>334</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>306</v>
+        <v>335</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>307</v>
+        <v>336</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>308</v>
+        <v>337</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>309</v>
+        <v>338</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>310</v>
+        <v>339</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>311</v>
+        <v>340</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9378,36 +10468,36 @@
         <v>32</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>312</v>
+        <v>341</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>313</v>
+        <v>342</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>314</v>
+        <v>343</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>315</v>
+        <v>344</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>316</v>
+        <v>345</v>
       </c>
       <c r="G2" s="10" t="s">
-        <v>317</v>
+        <v>346</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>318</v>
+        <v>347</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>319</v>
+        <v>348</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>320</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>321</v>
+        <v>350</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -9421,7 +10511,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>322</v>
+        <v>351</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -9435,7 +10525,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>323</v>
+        <v>352</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -9449,7 +10539,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>324</v>
+        <v>353</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -9463,7 +10553,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>325</v>
+        <v>354</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -9477,7 +10567,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>326</v>
+        <v>355</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -9491,7 +10581,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>327</v>
+        <v>356</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -9505,7 +10595,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>328</v>
+        <v>357</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -9553,25 +10643,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>329</v>
+        <v>358</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>330</v>
+        <v>359</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>331</v>
+        <v>360</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>332</v>
+        <v>361</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>333</v>
+        <v>362</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>334</v>
+        <v>363</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>335</v>
+        <v>364</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9579,27 +10669,27 @@
         <v>32</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>336</v>
+        <v>365</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>337</v>
+        <v>366</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>338</v>
+        <v>367</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>339</v>
+        <v>368</v>
       </c>
       <c r="F2" s="12" t="s">
         <v>227</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>340</v>
+        <v>369</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>341</v>
+        <v>370</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -9610,7 +10700,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>342</v>
+        <v>371</v>
       </c>
       <c r="B4" s="17"/>
       <c r="C4" s="17"/>
@@ -9621,7 +10711,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>343</v>
+        <v>372</v>
       </c>
       <c r="B5" s="17"/>
       <c r="C5" s="17"/>
@@ -9632,7 +10722,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>344</v>
+        <v>373</v>
       </c>
       <c r="B6" s="17"/>
       <c r="C6" s="17"/>
@@ -9643,7 +10733,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>345</v>
+        <v>374</v>
       </c>
       <c r="B7" s="17"/>
       <c r="C7" s="17"/>
@@ -9654,7 +10744,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>346</v>
+        <v>375</v>
       </c>
       <c r="B8" s="17"/>
       <c r="C8" s="17"/>
@@ -9665,7 +10755,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>347</v>
+        <v>376</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -9676,7 +10766,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>348</v>
+        <v>377</v>
       </c>
       <c r="B10" s="17"/>
       <c r="C10" s="17"/>
@@ -9687,7 +10777,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>349</v>
+        <v>378</v>
       </c>
       <c r="B11" s="17"/>
       <c r="C11" s="17"/>
@@ -9698,7 +10788,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>350</v>
+        <v>379</v>
       </c>
       <c r="B12" s="17"/>
       <c r="C12" s="17"/>
@@ -9709,7 +10799,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>351</v>
+        <v>380</v>
       </c>
       <c r="B13" s="17"/>
       <c r="C13" s="17"/>
@@ -9720,7 +10810,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>352</v>
+        <v>381</v>
       </c>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -9731,7 +10821,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>353</v>
+        <v>382</v>
       </c>
       <c r="B15" s="17"/>
       <c r="C15" s="17"/>
@@ -9742,7 +10832,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>354</v>
+        <v>383</v>
       </c>
       <c r="B16" s="17"/>
       <c r="C16" s="17"/>
@@ -9753,7 +10843,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>355</v>
+        <v>384</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="17"/>
@@ -9764,7 +10854,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>356</v>
+        <v>385</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="17"/>
@@ -9775,7 +10865,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>357</v>
+        <v>386</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="17"/>
@@ -9786,7 +10876,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>358</v>
+        <v>387</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -9797,7 +10887,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>359</v>
+        <v>388</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="17"/>
@@ -9808,7 +10898,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>360</v>
+        <v>389</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="17"/>

</xml_diff>